<commit_message>
LEARNT XLOOKUP, VLOOKUP AND INDEX-MATCH
</commit_message>
<xml_diff>
--- a/Excel+LAB+4+Dataset_Dmart_Cleaning_Structuring.xlsx
+++ b/Excel+LAB+4+Dataset_Dmart_Cleaning_Structuring.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Documents\AdvExcel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43E3D6EE-623B-4CFF-B918-3C86AF698166}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA3DA336-070A-4D7E-A59B-07EEF0191C15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DMart_Data_Set" sheetId="1" r:id="rId1"/>
@@ -18,9 +18,10 @@
     <sheet name="CustomList2" sheetId="4" r:id="rId3"/>
     <sheet name="CustomData" sheetId="5" r:id="rId4"/>
     <sheet name="LOOKUPfunctions" sheetId="10" r:id="rId5"/>
-    <sheet name="Sheet1" sheetId="6" r:id="rId6"/>
-    <sheet name="Sheet2" sheetId="7" r:id="rId7"/>
-    <sheet name="Sheet3" sheetId="9" r:id="rId8"/>
+    <sheet name="HLOOKUP" sheetId="11" r:id="rId6"/>
+    <sheet name="Sheet1" sheetId="6" r:id="rId7"/>
+    <sheet name="Sheet2" sheetId="7" r:id="rId8"/>
+    <sheet name="Sheet3" sheetId="9" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="Orders">DMart_Sales_Data[OrderID]</definedName>
@@ -38,14 +39,14 @@
       </xcalcf:calcFeatures>
     </ext>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId9" roundtripDataChecksum="gT5L9Uh5Mkce+NjaHPxVAbIJlDW9RbqkjfO6mNdsl18="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId10" roundtripDataChecksum="gT5L9Uh5Mkce+NjaHPxVAbIJlDW9RbqkjfO6mNdsl18="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3769" uniqueCount="689">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3789" uniqueCount="698">
   <si>
     <t>Region</t>
   </si>
@@ -2163,6 +2164,33 @@
   <si>
     <t>Using Index-Match</t>
   </si>
+  <si>
+    <t>Jan</t>
+  </si>
+  <si>
+    <t>Feb</t>
+  </si>
+  <si>
+    <t>Mar</t>
+  </si>
+  <si>
+    <t>Apr</t>
+  </si>
+  <si>
+    <t>Cost</t>
+  </si>
+  <si>
+    <t>Travel</t>
+  </si>
+  <si>
+    <t>Profit</t>
+  </si>
+  <si>
+    <t>Month</t>
+  </si>
+  <si>
+    <t>Using VLOOKUP</t>
+  </si>
 </sst>
 </file>
 
@@ -2172,11 +2200,18 @@
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="165" formatCode="&quot;₹&quot;\ #,##0.00"/>
   </numFmts>
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="27" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -2820,77 +2855,77 @@
   </borders>
   <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="104">
+  <cellXfs count="106">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="9" xfId="3" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="9" xfId="4" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="10" xfId="3" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="10" xfId="4" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="9" xfId="3" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="9" xfId="4" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="10" xfId="3" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="10" xfId="4" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
@@ -2899,63 +2934,63 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="20" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="20" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="20" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="20" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="14" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="3" fontId="22" fillId="16" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="23" fillId="16" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="12" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
@@ -2966,28 +3001,30 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="26" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="18" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="40% - Accent3" xfId="3" builtinId="39"/>
@@ -49393,7 +49430,7 @@
       <c r="Y1000" s="1"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="8" type="noConversion"/>
+  <phoneticPr fontId="9" type="noConversion"/>
   <conditionalFormatting sqref="E1:F1048576">
     <cfRule type="top10" dxfId="3" priority="2" bottom="1" rank="10"/>
     <cfRule type="top10" dxfId="2" priority="3" rank="10"/>
@@ -49882,7 +49919,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="13" type="noConversion"/>
+  <phoneticPr fontId="14" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -50922,7 +50959,7 @@
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="D3:E14">
     <sortCondition ref="D3:D14" customList="January,February,March,April,May,June,July,August,September,October,November,December"/>
   </sortState>
-  <phoneticPr fontId="13" type="noConversion"/>
+  <phoneticPr fontId="14" type="noConversion"/>
   <conditionalFormatting sqref="E3:E14">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThan">
       <formula>50000</formula>
@@ -51228,7 +51265,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="13" type="noConversion"/>
+  <phoneticPr fontId="14" type="noConversion"/>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C13:C15 C19" xr:uid="{EA1DFDD7-EA19-432F-9135-1EEE37691A5F}">
       <formula1>$A$2:$A$9</formula1>
@@ -51239,6 +51276,198 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FABEF5C-D0AD-491C-B800-CFAE06B8007C}">
+  <dimension ref="A2:F14"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="27"/>
+      <c r="B2" s="25" t="s">
+        <v>689</v>
+      </c>
+      <c r="C2" s="25" t="s">
+        <v>690</v>
+      </c>
+      <c r="D2" s="25" t="s">
+        <v>691</v>
+      </c>
+      <c r="E2" s="25" t="s">
+        <v>692</v>
+      </c>
+      <c r="F2" s="25" t="s">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="25" t="s">
+        <v>693</v>
+      </c>
+      <c r="B3" s="27">
+        <v>100</v>
+      </c>
+      <c r="C3" s="27">
+        <v>585</v>
+      </c>
+      <c r="D3" s="27">
+        <v>333</v>
+      </c>
+      <c r="E3" s="27">
+        <v>745</v>
+      </c>
+      <c r="F3" s="27">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="25" t="s">
+        <v>694</v>
+      </c>
+      <c r="B4" s="27">
+        <v>100</v>
+      </c>
+      <c r="C4" s="27">
+        <v>500</v>
+      </c>
+      <c r="D4" s="27">
+        <v>600</v>
+      </c>
+      <c r="E4" s="27">
+        <v>700</v>
+      </c>
+      <c r="F4" s="27">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="25" t="s">
+        <v>577</v>
+      </c>
+      <c r="B5" s="27">
+        <v>2000</v>
+      </c>
+      <c r="C5" s="27">
+        <v>7000</v>
+      </c>
+      <c r="D5" s="27">
+        <v>8000</v>
+      </c>
+      <c r="E5" s="27">
+        <v>6000</v>
+      </c>
+      <c r="F5" s="27">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="25" t="s">
+        <v>695</v>
+      </c>
+      <c r="B6" s="27">
+        <v>400</v>
+      </c>
+      <c r="C6" s="27">
+        <v>500</v>
+      </c>
+      <c r="D6" s="27">
+        <v>300</v>
+      </c>
+      <c r="E6" s="27">
+        <v>300</v>
+      </c>
+      <c r="F6" s="27">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E9" s="105" t="s">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B10" s="25" t="s">
+        <v>696</v>
+      </c>
+      <c r="C10" s="25" t="s">
+        <v>692</v>
+      </c>
+      <c r="E10" s="25" t="s">
+        <v>696</v>
+      </c>
+      <c r="F10" s="25" t="s">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B11" s="25" t="s">
+        <v>577</v>
+      </c>
+      <c r="C11" s="27">
+        <f>HLOOKUP($C$10,$A$2:$F$6,MATCH(B11,$A$2:$A$6,0),FALSE)</f>
+        <v>6000</v>
+      </c>
+      <c r="E11" s="25" t="s">
+        <v>577</v>
+      </c>
+      <c r="F11" s="27">
+        <f>VLOOKUP(E11,$A$2:$F$6,MATCH($F$10,$A$2:$F$2,0),FALSE)</f>
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B12" s="25" t="s">
+        <v>694</v>
+      </c>
+      <c r="C12" s="27">
+        <f>HLOOKUP($C$10,$A$2:$F$6,MATCH(B12,$A$2:$A$6,0),FALSE)</f>
+        <v>700</v>
+      </c>
+      <c r="E12" s="104" t="s">
+        <v>695</v>
+      </c>
+      <c r="F12" s="27">
+        <f t="shared" ref="F12:F14" si="0">VLOOKUP(E12,$A$2:$F$6,MATCH($F$10,$A$2:$F$2,0),FALSE)</f>
+        <v>200</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B13" s="104" t="s">
+        <v>693</v>
+      </c>
+      <c r="C13" s="27">
+        <f>HLOOKUP($C$10,$A$2:$F$6,MATCH(B13,$A$2:$A$6,0),FALSE)</f>
+        <v>745</v>
+      </c>
+      <c r="E13" s="104" t="s">
+        <v>693</v>
+      </c>
+      <c r="F13" s="27">
+        <f t="shared" si="0"/>
+        <v>222</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B14" s="104" t="s">
+        <v>695</v>
+      </c>
+      <c r="C14" s="27">
+        <f>HLOOKUP($C$10,$A$2:$F$6,MATCH(B14,$A$2:$A$6,0),FALSE)</f>
+        <v>300</v>
+      </c>
+      <c r="E14" s="104" t="s">
+        <v>694</v>
+      </c>
+      <c r="F14" s="27">
+        <f t="shared" si="0"/>
+        <v>900</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="9" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CE4AEB2-99B1-4F87-956C-8EC68CB27B81}">
   <dimension ref="A1:A12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -51297,13 +51526,13 @@
       <c r="A12" s="93"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="13" type="noConversion"/>
+  <phoneticPr fontId="14" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A885D05-95FE-496B-A37F-A62FFC99FFE7}">
   <dimension ref="A1:A12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -51372,12 +51601,12 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="13" type="noConversion"/>
+  <phoneticPr fontId="14" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F9E0CCF-A626-41AD-8D97-0A4946B1AEFD}">
   <dimension ref="A1:A12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -51446,7 +51675,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="13" type="noConversion"/>
+  <phoneticPr fontId="14" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>